<commit_message>
fix(lgo): pas-à-pas vérifiés par 4 audits — LGPI sans prix dit clairement, mail propre au catalogue, « Si l'import bloque » sur les 8 PDF, captures entières, plus de « remise », garde Escale/OPSO, iPhone 16 px/44 px
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/crm/v2/lgo/integral-top200-pharmaland.xlsx
+++ b/crm/v2/lgo/integral-top200-pharmaland.xlsx
@@ -434,7 +434,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -451,7 +451,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>PRIX REMISE HT</t>
+          <t>PRIX NET HT</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">

</xml_diff>